<commit_message>
Auto: Week 24/2026 data extracted from PDFs
</commit_message>
<xml_diff>
--- a/Gulf_Dashboard_W24_2026.xlsx
+++ b/Gulf_Dashboard_W24_2026.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 24 Progress" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discipline Detail" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W24" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -54,8 +55,12 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -87,6 +92,11 @@
         <fgColor rgb="00FFC000"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE0E0"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -114,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -157,6 +167,15 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5679,4 +5698,1399 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>PRJ ID</t>
+        </is>
+      </c>
+      <c r="B1" s="15" t="inlineStr">
+        <is>
+          <t>Project Name</t>
+        </is>
+      </c>
+      <c r="C1" s="15" t="inlineStr">
+        <is>
+          <t>PDF Found</t>
+        </is>
+      </c>
+      <c r="D1" s="15" t="inlineStr">
+        <is>
+          <t>Concerns</t>
+        </is>
+      </c>
+      <c r="E1" s="15" t="inlineStr">
+        <is>
+          <t>Activities</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="16" t="inlineStr">
+        <is>
+          <t>PRJ-001</t>
+        </is>
+      </c>
+      <c r="B2" s="16" t="inlineStr">
+        <is>
+          <t>LNG Terminal (GMTP)</t>
+        </is>
+      </c>
+      <c r="C2" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D2" s="16" t="inlineStr">
+        <is>
+          <t>Unsafe Lifting Practice and Non- CMG deviated from the approved lifting procedure by performing multiple-
+GMTP-PCC-SHE-CAR-035 compliance with Approved Lifting 11 Jun 2026 item lifting (4 items in one lift) instead of single-item lifting. This unsafe Ongoing
+Plan at ISB building practice introduces significant hazards
+7.4 SHE NCR Status
+Doc No. Description Issue date Root cause Status
+M11 Pro PEC 17 Jun, 2026 5 Jun, 2026
+Vendor/ Subcontractor
+M12 Con CAZ Start Foundation Work for Jetty Control Building 17 Jul, 2026 30 Apr, 2026 30 Apr, 2026 6 May, 2026 5 Jun, 2026
+Chipping of Pile Head of LNG Tank2 completed
+M12 Con PEC 17 Jul, 2026 21 Feb, 2026
+(including Pile Integrity Test)
+M12 Con PEC Column for LNG Tank2 completed 17 Jul, 2026 4 Mar, 2026
+Issued PO for BOG Recondense and Truck loading confirm
+M12 Pro PEC 17 Jul, 2026 27 May, 2026
+received from Vendor/Subcontractor
+M12 Con PEC Start base slab work at LNG Tank2 area 17 Jul, 2026 22 Jan, 2026
+Issued PO for Pressure Vessels confirm received from
+M12 Eng PEC Issued Plot Plan IFC 17 Jul, 2026 13 Mar, 2026
+M12 Eng PEC Issued Above Ground Piping MTO for Construction 17 Jul, 2026 2 Apr, 2026
+M12 Eng PEC Issued Cryogenic Piping Supports MTO for Construction 17 Jul, 2026 2 Apr, 2026</t>
+        </is>
+      </c>
+      <c r="E2" s="16" t="inlineStr">
+        <is>
+          <t>- GMTP/PMC/PCC management mass TBT and safety share was held on 17 Jun 2026. - GMTP/PMC/PCC management TBT and safety share on 25 June 2026.
+- SHE/EIA weekly audit was held on 17 Jun 2026. - SHE/EIA weekly audit on 1 Jul 2026.
+- Big cleaning day on 13 Jun 2026. - Big cleaning day every Saturday.
+Security Security
+- Provided temporary security guard for control personal, vehicle and material at site main gate 24
+- Strictly control personnel and vehicle gate pass, check the entrance and exit of materials and hours.
+equipment into and out of the projectarea 24/7.(Night shift patrols every 1 hour)
+EIA/EHIA EIA/EHIA
+- Dry-run EIA/EHIA Committee Meeting on 16 Jun 2026
+- Worker camp monthly audit and concrete dumping area audit on 17 Jun 2026 - EIA/EHIA Committee Meeting on 24 Jun 2026
+Issue for Issue for Document Class
+Approval Construction Z X Y
+General 0 0 0 0 0
+Process 0 0 0 0 0
+Mechanical 0 0 0 0 0
+Mechanical (Tank) 0 0 0 0 0
+Piping 0 0 0 0 0
+Electrical 0 0 0 0 0
+Instrument 0 6 6 0 0
+Civil (BOP) 0 0 0 0 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t>PRJ-002</t>
+        </is>
+      </c>
+      <c r="B3" s="16" t="inlineStr">
+        <is>
+          <t>GOE2-NWT3</t>
+        </is>
+      </c>
+      <c r="C3" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D3" s="16" t="inlineStr">
+        <is>
+          <t>Complaint from Villagers:
+➢ To expedite manpower, machine, scaffolding and tools for install mounting and PV module.
+115kV Substation:
+➢ To expedite fabricate roof structure.
+115kV Transmission line:
+➢ Construction work can start after Permit approval.</t>
+        </is>
+      </c>
+      <c r="E3" s="16" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>PRJ-003</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>GSPG-PTN</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D4" s="16" t="inlineStr">
+        <is>
+          <t>No Description Date Location Company
+A fire caused by suspected arson occurred in Laydown Area 2,
+resulting in extensive damage to PV modules. Jun 15, 2026 Laydown 2 512 boxes GUE
+Complaint from Villagers:
+Pre-Civil work :
+➢ Site Incident - Security Issue, which may impact project schedule.
+➢ To expedite the delayed Pre-Civil work to be complete and handover to C&amp;E work.
+➢ To expedite Electrical work and increase manpower.
+➢ To expedite civil work for unit sub.
+➢ Manpower not on site as Plan
+➢ The rainy season may cause waterlogging across the site, which could decrease site progress.
+115kV Substation:
+➢ To expedite Electrical work.
+115kV Transmission line:
+➢ To expedite the delayed foundation work ,concrete pole and top pole installation work.
+115kV add bay:
+➢ To expedite the delayed Civil work.</t>
+        </is>
+      </c>
+      <c r="E4" s="16" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>PRJ-004</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>GSPG-STN</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Complaint from Villagers:
+➢ Residents living in the vicinity of the project have reported cracks in their houses.
+➢ Chusin Co., Ltd. has requested that the project urgently resolve the issue of rainwater from the project draining into nearby areas.
+3J Thailand Pre-Civil work :
+GUE PV farm:
+➢ To expedite the mobilization of the additional manpower for the Unit substation.
+➢ To expedite the mobilization of the additional manpower for the Electrical works.
+SIEMENS 115kV Substation:
+➢ To expedite the mobilization of the additional manpower for the Civil works.
+PEA&amp;FEC 115kV Transmission line:
+➢ To expedite start Electrical work.
+PEA&amp;FEC Communication/Fiber :</t>
+        </is>
+      </c>
+      <c r="E5" s="16" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>PRJ-005</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>LNE</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D6" s="16" t="inlineStr"/>
+      <c r="E6" s="16" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>PRJ-006</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>SSE</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Total Indirect Workforce 70 60 +10
+Total Direct Workforce 271 203 +68</t>
+        </is>
+      </c>
+      <c r="E7" s="16" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>PRJ-007</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>SDCE</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>C&amp;E Construction:
+115kV Substation:
+115kV Transmission Line:
+• Project progress is delayed due to insufficient manpower and heavy equipment — immediate mobilization of additional teams required to
+recover schedule.
+Addbay Tha Yang Substation:
+GIS Substation:</t>
+        </is>
+      </c>
+      <c r="E8" s="16" t="inlineStr">
+        <is>
+          <t>Civil work Civil work
+➢ Continue permanent fence work. ➢ Continue permanent fence work.
+➢ Continue steel structure installation at transformer ➢ Continue steel structure installation at transformer
+station and BESS area. station and BESS area.
+Electrical work Electrical work
+➢ Continue Mounting and PV panel installation. ➢ Continue Mounting and PV panel installation.
+➢ Ground cable PV area installation. ➢ Ground cable PV area installation.
+➢ Continue DC cable and LV AC installation. ➢ Continue DC cable and LV AC installation.
+➢ Continue string inverter installation. ➢ Continue SAT/Individual work.
+➢ Continue SAT/Individual work. ➢ Continue MV Cable installation.
+➢ Continue MV Cable installation. ➢ Continue Cable test and IV Curve test.
+➢ Start Cable test and IV Curve test.
+➢ Plastering work for admin building completed. ➢ Continue ceramic tile work for admin building.
+➢ Start ceramic tile work for admin building. ➢ Continue architecture work.
+➢ Start vinyl tile work. ➢ Start Crush stone at SWYD installation.
+➢ Continue architecture work.
+➢ MV cable trench completed. Electrical work
+➢ External cable wiring completed.
+Electrical work ➢ Protection relay panel installation completed.
+➢ Continue external cable pulling. ➢ AC, DC panel installation completed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>PRJ-009</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>AL1 (Alpha 1)</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>• The tree cutting works of local villager land AL1 no.062 not yet completed. This affect the site
+clearing, road construction and further extend the duration of Extension of Time (EoT).
+• Soil disposal area insufficient and will be impacted as below:
+West Route = Expected to be impacted with concrete pump position for WTG06.
+East Route = Expected to be impacted by mid June.
+Route to Substation = Expected to be impacted first week of July.
+• East Route: The highlight area not yet compensated with landowner, but trees cutting already
+• Remaining trees in WTG07 area
+The remaining trees obstruct the road toe slope and
+soil disposal area.
+Remaining Trees
+• Rubber trees = 9 Ea.
+• Oil palm trees = 4 Ea.
+• Remaining trees and rubber rolling house along road of east route
+The remaining trees and rubber rolling house obstruct the slope protection and toe slope.
+• Durian trees = 14 Ea., Rambutan tree = 1 Ea., oil palm trees = 3 Ea.
+• Rubber rolling house = 1 Ea.
+• Remaining trees along road of east route
+The remaining trees obstruct the road slope protection.
+• Durian tree = 1 Ea.</t>
+        </is>
+      </c>
+      <c r="E9" s="16" t="inlineStr">
+        <is>
+          <t>➢ Road excavation at east route.
+➢ Backfill and Compaction for subgrade at west route.
+➢ Continue rock breaking at east route.
+➢ Continue box culvert construction at route to substation.
+➢ Continue excavation hardstand for WTG03.
+➢ Continue excavation foundation for WTG07.
+➢ Continue TSA access west route.
+➢ Rebar cutting, bending for WTG06 foundation.
+➢ DCPT for WTG01, WTG02, WTG03 foundation
+➢ Backfill and compaction for WTG06 foundation.
+➢ Plate Bearing test and pouring lean concrete for WTG08 foundation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>PRJ-010</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>AL2 (Alpha 2)</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
+        <is>
+          <t>Overall Progress
+Engineering
+Procurement
+Construction -
+at Thongmongkol subdistrict meeting room 1. Construction trucks transporting equipment and materials caused soil
+spillage on public roads, resulting in slippery surfaces and increased
+• Participants
+accident risk for local residents.
+• Mayor of Thong Mongkhon Subdistrict Administrative
+Soil and rocks from construction activities have fallen into agricultural
+Organization (SAO) and SAO officers
+areas, causing crop damage and posing potential risks to farmers.
+• Gulf Team &amp; Community Relations (CR)
+Excavation works for pole installation were carried out without proper
+• Interlink
+coordination or verification of existing utility alignments, leading to damage
+• VAP / CK to the village water supply pipeline and disruption of water services to the
+• Affected villagers (Moo 5 and Moo 10)
+Traffic and Transportation (Moo 5 – Soi Sam Phi Nong)
+Construction trucks transporting equipment and materials have caused soil spillage on public roads,</t>
+        </is>
+      </c>
+      <c r="E10" s="16" t="inlineStr">
+        <is>
+          <t>➢ Continue Cut and Fill for Subgrade layer North A ,Central A, Central B and South
+➢ Continue Pipe and Box culvert
+- South STA. 1+410 , 1+480 and STA. 1+710
+➢ Start 33kV Pole Installation at Service Road
+Actual Completed Deviation
+Fri Sat Sun Mon Tue Wed Thu Fri Sat Sun Mon Tue Wed Thu Fri Sat Sun Mon Tue Wed Thu Fri Sat Sun Mon Tue Wed Thu
+Start Finish
+6/5 6/6 6/7 6/8 6/9 6/10 6/11 6/12 6/13 6/14 6/15 6/16 6/17 6/18 6/19 6/20 6/21 6/22 6/23 6/24 6/25 6/26 6/27 6/28 6/29 6/30 7/1 7/2
+1 North A ( STA.1+400 - STA.4+667 )
+Plan 17-Apr 11-Jun 7.5% 7.5% 7.5% 7.5% 7.5% 7.5% 5%
+1 CUT &amp; FILL BEFORE COMPACTED SUBGRADE STA.2+500 -STA.3+000
+Actual 17-Apr 11-Jun 50.0% 0.0% 7.5% 7.5% 5% 7.5% 7.5% 7.5% 7.5%
+Plan 17-Apr 25-Jun 7.5% 7.5% 7.5% 7.5% 7.5% 7.5% 5% 7.5% 7.5% 7.5% 7.5% 7.5% 7.5% 5% 7.5% 7.5% 7.5% 7.5% 7.5% 7.5% 5%
+2 CUT &amp; FILL BEFORE COMPACTED SUBGRADE STA.3+000 -STA.3+500
+Actual 17-Apr 50.0% 0.0% 7.5% 7.5% 5% 5% 7.5% 7.5% 5.0% 7.5% 7.5% 7.5% 7.5% 7.5% 7.5% 5%
+Plan 15-Apr 9-Jul 7.5% 7.5% 7.5% 7.5% 7.5% 7.5% 5% 7.5% 7.5% 7.5% 7.5% 7.5% 7.5% 5%
+2 CUT &amp; FILL BEFORE COMPACTED SUBGRADE STA.3+500 -STA.4+000
+Actual 15-Apr 50.0% 0.0% 5% 5% 5% 5% 7.5% 7.5% 7.5% 7.5% 7.5% 7.5% 7.5% 7.5% 7.5% 5%
+Plan 29-May 2-Jul 7.5% 7.5% 7.5% 7.5% 7.5% 7.5% 5% 7.5% 7.5% 7.5% 7.5% 7.5% 7.5% 5% 7.5% 7.5% 7.5% 7.5% 7.5% 7.5% 5% 7.5% 7.5% 7.5% 7.5% 7.5% 7.5% 5%
+3 CUT &amp; FILL BEFORE COMPACTED SUBGRADE STA.4+000 -STA.4+500</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>PRJ-011</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>ECE</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>occurs in areas where road construction or drainage works are being
+carried out. Barricades and signage are often removed to allow access,
+but they are not reinstalled after the work is completed.
+• 22kV Detour Line obstructs blade transportation at 4 locations (Route 212 → ECE project site), which may impact the
+transportation of the wind turbine blades.
+• At certain WTG locations, the Hardstand (TSA) level does not correspond with the road level (CBOP), which may have an
+adverse impact on the transportation and installation of the wind turbine components.
+115kV Substation
+115kV Transmission Line</t>
+        </is>
+      </c>
+      <c r="E11" s="16" t="inlineStr">
+        <is>
+          <t>➢ Continue to road base course compaction work.
+➢ Continue to excavation and installation for 33kV Pole.
+➢ Continue to excavation work for drainage system.
+➢ Continue to excavation work.
+➢ Continue to rebar installation.
+➢ Plan to pouring lean concrete at WTG - 04 on 20 June 2026.
+➢ Continue to site preparation (Earth Work).
+➢ Continue foundation concrete pouring work.
+➢ Continue foundation rebar and formwork installation work.
+➢ Continue foundation excavation work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>PRJ-013</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>GCE</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t>➢ GCE-001-C-022-UAE-201_Bunker pit ground floor framing plan EL +0.25 s the concern about the increased slope of 20 cm correct?
+Concern (delay)
+The drawing needs to be fixed urgently within endof June
+Affect to planslab ground floor
+Co-ordinated with civil team EPC and OE for follow up
+➢ GCE-001-E-018-CYE-001_FIRE ALARM SYSTEM GENERAL CABLE ROUTING There are no details about the pipe laying depth
+STECON is unable to plan for the excavation.
+Follow up with EPC &amp; STECON expediting to get the depth of rout line within mid of June .
+EPC &amp; STECON acknowledge.
+Summary of Safety Weekly Audit issues
+Total Issues 3 8 9 5
+since 03 Apr 2026 - Present 21-May 26-May 4-Jun 11-Jun 18-Jun
+(Every Tuesday morning)
+Open Closed
+Safety Audit issue Status Chart
+4 Environmental Impact Assessment Committee meeting. -Environment Impact At least SM ,CR and -
+Done 27 May 2026
+Assessment Committee twice a year SSHE
+5 Provide support for activities as requested by the community -School ,Government As CR -
+and Government. Agencies ,temple appropriate. Done</t>
+        </is>
+      </c>
+      <c r="E12" s="16" t="inlineStr">
+        <is>
+          <t>Key Lookahead milestone:
+Commissioning 0.00% 0.00% -
+Pre-conditions required:
+Total Man-Hours 335,193 Area of Concern:
+Permanence fence drawing
+Transformer FOUNDATION PLAN AND DETAIL drawing not yet.
+Zijian boiler installation team QA/QC Urgent resignation 2 person
+start Construction phase (Excuvation work) on 26/12/2025 4. STCEON's workforce increase did not go according to plan.
+Issue to request HO support:
+SM EPC is urging its EPC design and engineering teams to provide the data.
+Safety &amp; Health:
+Management site walkdown
+Toolbox talk activity
+Safety induction training to new contractors​
+Weekly Inspect Safety​
+Weekly Random Alc. Test
+Fire and Evacuate drill on 24 Jun 2026
+Environment &amp; CoP:
+Road cleaning (Campsite STECON/IEAT Road)
+Water spray to reduce dust</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>PRJ-014</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>GSE</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>Bunker and surrounding: Foundation up to ground (including the surrounding room, underground grounding system).
+Boiler : Boiler steel structure.
+Flue gas treatment : Foundation work.
+STG &amp; ECB : Foundation up to ground (including the surrounding room, underground grounding system).
+Tipping hall: Pilling work and foundation.
+Concern (delay)
+Delay finish of bunker foundations up to ground level. Target on PMS 07 May 2026.
+Delay finish of STG foundations up to ground level. Target on PMS 25 May 2026.
+CEEC/STECON prepare catch-up plan for bunker and boiler foundation up to ground level
+CEEC/STECON will increase man power more than plan
+- This week (Finished : 1 , Remaining : 2)
+- Total (Finished : 32 , Remaining : 2)
+NO RFC , NO NCR
+7 Stakeholder Engagement Plan Continue as plan
+8 SHE Plan for counting manpower working at site There will be generated counting manpower data report the first time on
+&lt;22 Jun 2026&gt;
+9 Status of EPC Foreigner staff and worker personal mandatory document Pending 27 prs. &lt;Plan to finish Jun 2026&gt;
+34 Safety Weekly Audit issue
+Total Issues
+(Since 2 Apr 2026 onwards)</t>
+        </is>
+      </c>
+      <c r="E13" s="16" t="inlineStr">
+        <is>
+          <t>Activities CC/SC (*)
+Plan Actual Diff. Plan Actual Diff. Acc.Plan
+% % % % % % %
+Engineering 10% 59.50% 42.02% -17.48% 67.58% 43.90% -23.68% 74.32%
+Procurement 40% 68.99% 65.43% -3.56% 71.12% 69.35% -1.77% 72.89%
+Construction 40% 11.51% 10.22% -1.29% 13.16% 10.70% -2.46% 14.29%
+Commissioning 10% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00%
+Overall 100% 38.15% 34.46% -3.69% 40.47% 36.41% -4.06% 42.30%
+5 Maximum Quantity of Heavy Machinery at Site Inspection as period
+and keep related document
+6 Summary of SHE Weekly Audit issues Walk down
+- This week (Finished : 1 , Remaining : 2)
+- Total (Finished : 32 , Remaining : 2)
+NO RFC , NO NCR
+7 Stakeholder Engagement Plan Continue as plan
+8 SHE Plan for counting manpower working at site There will be generated counting manpower data report the first time on
+&lt;22 Jun 2026&gt;
+9 Status of EPC Foreigner staff and worker personal mandatory document Pending 27 prs. &lt;Plan to finish Jun 2026&gt;
+Safety &amp; Health:
+• Safety Toolbox Talk before starting work and Mass Toolbox Talk and counting manpower</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>PRJ-015</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>KKE</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D14" s="16" t="inlineStr">
+        <is>
+          <t>311-314 Refuse Bunker Super structure up to 35.5m elevation 9 May 26 23 Nov 26 Delay Start
+325-326 Tipping hall Foundation up to ground (Include piling work) 1 Feb 26 9 Jul 26 8 Feb 26 On going
+327 Tipping hall Super structure up to 13m elevation 10 Jul 26 19 Oct 26
+330-335 Boiler Island &amp; Auxiliary Equipment Foundation 5 Nov 25 14 Jul 26 8 Jan 26 On going
+346 Steam Turbine Generator &amp; Electrical Construction 18 Feb 26 3 Mar 27 8 Feb 26 On going
+408 Holding Pond and Emergency PondConstruction 23 May 26 20 Nov 26
+14 Boiler Arrival at site 12 Jun 26 12 Jun 26
+11 Incinerator Arrival at site 8 May 26 8 May 26 3 May 26 5 May 26 Completed
+15 Steam turbine Arrival at site 2 Oct 26 2 Oct 26
+62- Producing qualified water (Water Receiving date) 23 Feb 27 8 Mar 27
+EPC has adjusted the PMS to Rev.H to make the plan consistent with the actual work
+Completion of Bunker building Ground slab
+Completion of Lift 2: Bunker wall +1.0 to +5.45 EL.
+Completed of Steel structure erection for Upper part Z1-Z6 at 11.3-41.6 m.
+Commencement of FGT equipment steel structure erection.
+Partial handover (civil works) of Switchgear room in the STG &amp; EC Building, including all related areas required for the installation of 22 kV and 11 kV switchgear and
+power cables.
+Unsuitable ground condition for 300T crawler crane assembly may affect upcoming steel structure erection activities.
+117 Safety Weekly Audit issue status by weekly
+Total Issues</t>
+        </is>
+      </c>
+      <c r="E14" s="16" t="inlineStr">
+        <is>
+          <t>Key Lookahead milestone: 1. Bunker building: Concrete pouring for Lift 2 Wall +1.0 to +5.45 EL
+Targeted by 28-29 Jun 26
+Boiler &amp; Incinerator Erection: Steel structure erection for Upper part Z1-Z3 at 11.3-41.6 m
+FGT: Clearance for FGT Equipment steel support structure erection.
+STG &amp; ECB: Foundation Up to ground
+The tower crane: installation Targeted by 27-Jun-26
+Balance of Plant: Commencement of piling works on 22-Jun-26
+Pre-conditions required: Unsuitable ground condition for 300T crawler crane assembly may affect
+upcoming steel structure erection activities.
+Area of Concern:
+Bunker, Boiler &amp; FGT Installation: Level 3 schedule update remains outstanding.
+HDPE fire fighting pipe: ASTM-compliant pipe is not available from local suppliers in Thailand and
+may need to be imported, which could extend procurement lead time and impact construction schedule
+Issue to request HO support: None
+Completed of Pile head treatment for Tipping hall area.
+Commencement of piling works for the Balance of Plant.
+Concern (delay).
+Unsuitable ground condition for 300T crawler crane assembly may affect upcoming steel structure erection activities.
+Expedite CEEC/HUASHI to carry out backfilling and soil compaction testing works to enable crawler crane access to the area
+Safety &amp; Health</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>PRJ-016</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>MKP</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Bunker Pit Wall to +5.45 EL
+Bunker Building ground level construction
+Boiler structure construction
+STG&amp;EC Building construction
+Underground Piping work
+Pile Driving for Tipping Area
+Duct bank and Cathodic protection installation
+Concern (delay)
+Late manufacturing for steel roof structure and cladding structure
+Accuracy of embedded plate installation
+Underground pipes are required long lead for fabrication and delivery from oversea manufacturer. (Steel pipe 24”&amp;28”)
+1 Duct bank and Cathodic protection drawing were not finalized
+2 Delay of Material purchasing.
+Follow-up CEEC/SEPEC to urgently conclude the detail of steel roof structure and cladding structure
+SEPEC/STECON are required to ensure embedded plates are installed at the correct elevation
+STECON proceed to purchasing and prepare catch-up plan
+1 Follow-up the detail drawing of Duct bank and Cathodic protection in Weekly meeting.
+2 Request CEEC to update purchasing status of Duct bank and Cathodic protection.
+49 Safety Weekly Audit issue status by weekly
+Total Issues</t>
+        </is>
+      </c>
+      <c r="E15" s="16" t="inlineStr">
+        <is>
+          <t>(12 Jun 26) (19 Jun 26)
+Activities CC/SC (*)
+Plan Actual Diff. Plan Actual Diff. Acc.Plan
+% % % % % % %
+Engineering 10% 44.31 40.39 -3.92 49.18 42.00 -7.18 53.60
+Procurement 40% 63.28 57.28 -6.00 65.88 63.65 -2.23 67.82
+Construction 40% 6.41 7.72 1.31 7.14 8.29 1.15 8.21
+Commissioning 10% 0 0 0 0 0 0 0
+Overall 100% 32.31 30.04 -2.27 34.13 32.98 -1.15 35.77
+Safety &amp; Health :
+• Conduct SafetyToolbox Talk before starting work.
+• Mass Safety Talk at Site Area
+• Management Walk Down every Friday (10.00 – 11.00)
+• HSE Weekly Audit every Wednesday (10.00-11.00)
+• HSE Weekly Meeting with Subcontractor every Wednesday (10.00-11.00)
+• Safety Induction Training for newcomers
+• Working at height Training
+Environment &amp; CoP :
+• Water spray at construction site
+• Temporary Wheel wash station</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>PRJ-017</t>
+        </is>
+      </c>
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>MPE</t>
+        </is>
+      </c>
+      <c r="C16" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D16" s="16" t="inlineStr">
+        <is>
+          <t>➢ Boiler foundation construction
+➢ Steam Turbine Generator &amp; Electrical Construction
+Concern (delay)
+Tasks that have started and those that have not yet started are behind schedule (PMS plan).
+Follow-up work with catch-up plan by daily.
+Expedite to EPC&amp; STECON increase manpower.
+Follow –up manpower with STECON in weekly and daily meeting.
+Expediting STECON to do work with catch-up plan by daily
+Plan to do parallel work .
+Safety Weekly Audit issue status by weekly
+Total Issues
+since 02 Apr 2026 - Present
+(Every Tuesday morning)
+21-May-26 28-May-26 4-Jun-26 11-Jun-26 18-Jun-26
+Safety Audit issue Status Chart Open Closed
+Open Closed
+and anxieties.
+Environmental Impact Assessment -Environment Impact Assessment At least twice SM ,CR and -
+Done 27 May 2026
+Committee meeting. Committee a year SSHE</t>
+        </is>
+      </c>
+      <c r="E16" s="16" t="inlineStr">
+        <is>
+          <t>Safety &amp; Health:
+Management site walkdown
+Toolbox talk activity
+Safety induction training to new contractors​
+Weekly Inspect Safety​
+Weekly Random Alc. Test
+Fire and Evacuate drill on 24 Jun 2026
+Environment &amp; CoP:
+Road cleaning (Campsite STECON/IEAT Road)
+Water spray to reduce dust
+Monitor noise during overtime work
+Activities CC/SC (*)
+Plan Actual Diff. Plan Actual Diff. Acc.Plan
+% % % % % % %
+Engineering 10.00% 40.82% 40.52% -0.30% 45.80% 42.11% -3.69% 49.27%
+Procurement 40.00% 44.72% 53.04% 8.32% 47.48% 54.24% 6.76% 50.28%
+Construction 40.00% 4.52% 5.83% 1.31% 4.85% 6.05% 1.20% 5.22%
+Commissioning 10.00% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00%
+Overall 100.00% 23.78% 27.60% 3.82% 25.51% 28.32% 2.81% 27.13%
+** The data cut off every Friday of week.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>PRJ-018</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>PFP</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Boiler foundation construction work.
+Steam Turbine Generator &amp; Electrical Construction work .
+Concern (Delay)
+Tasks that have started and those that have not yet started are behind schedule (PMS plan)
+• Follow-up work with catch-up plan by daily
+• Follow –up manpower with STECON in daily meeting
+• Expediting STECON to do work with catch-up plan by daily
+• Plan to do parallel work and reduce duration time some step of work.
+Safety Weekly Audit issue status by weekly
+Total Issues
+since 02 Apr 2026 - Present 20
+(Every Tuesday morning)
+21-May-26 29-May-26 4-Jun-26 11-Jun-26 18-Jun-26
+Open Closed
+Safety Audit issue Status Chart
+and anxieties.
+Environmental Impact Assessment -Environment Impact Assessment At least twice SM ,CR and -
+Done 27 May 2026
+Committee meeting. Committee a year SSHE
+Provide support for activities as requested -School ,Government Agencies ,temple As CR -</t>
+        </is>
+      </c>
+      <c r="E17" s="16" t="inlineStr">
+        <is>
+          <t>Safety &amp; Health:
+Management site walkdown
+Toolbox talk activity
+Safety induction training to new contractors​
+Weekly Inspect Safety​
+Weekly Random Alc. Test
+Fire and Evacuate drill on 24 Jun 2026
+Environment &amp; CoP:
+Road cleaning (Campsite STECON/IEAT Road)
+Water spray to reduce dust
+Monitor noise during overtime work
+Activities CC/SC (*)
+Plan Actual Diff. Plan Actual Diff. Acc.Plan
+% % % % % % %
+Engineering 10.00% 44.31% 40.14% -4.17% 49.18% 42.26% -6.92% 53.60%
+Procurement 40.00% 63.28% 57.28% -6.00% 65.88% 63.65% -2.23% 67.82%
+Construction 40.00% 6.41% 6.41% 0.00% 7.14% 6.61% -0.53% 8.21%
+Commissioning 10.00% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00%
+Overall 100.00% 32.31% 29.49% -2.82% 34.13% 32.33% -1.80% 35.77%
+** The data cut off every Friday of week.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>PRJ-019</t>
+        </is>
+      </c>
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>PKP</t>
+        </is>
+      </c>
+      <c r="C18" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D18" s="16" t="inlineStr">
+        <is>
+          <t>Completion of Bunker Building Concrete pouring Lift 1 Wall -5.7 to +1.0 EL ; (First step is to pour concrete up to kicker level on 3-4 Jul ; the second step is
+to pour the concrete up to +1.00 EL on 14-15 Jul
+CEEC/STECON will hand over the main 8 column pedestals (excluding the ground base slab) of the Boiler on 13-JUL- 2026 for HUASHI to perform
+the first lift of the steel structure on 14-JUL-2026. The remaining 4 column pedestals in the boiler area must be handed over to Huashi within 7 days
+on 20-JUL-2026 of the handover of the above columns.
+Partial handover (civil works) of Switchgear room in the STG &amp; EC Building, including all related areas required for the installation of 22 kV and 11 kV
+switchgear and power cables.
+Concern(delay)
+Increase Manpower up to 200 within June 2026
+Limited site access roads may impact construction productivity and material logistics.
+Site to Monitor Increasing of Manpower
+The Owner coordinated with CEEC and STECON to find a solution.
+57 Safety Weekly Audit issue status by weekly
+Total Issues 10
+Since 25 Jan 2026
+Safety Weekly Audit issue Status Chart
+Open Closed
+Before After
+Cement residuewas found Already improved.
+lying onthe ground in an</t>
+        </is>
+      </c>
+      <c r="E18" s="16" t="inlineStr">
+        <is>
+          <t>Key Lookahead milestone:
+Bunker Building : is under review by CEEC and expected to be submitted next week
+Boiler island area : STECON hand over to Huashi by 13-Jul-26
+STG&amp;ECB up to ground is under review by CEEC and expected to be submitted next week.
+Area of Concern:
+Increase Manpower up to 200 within June 2026
+Bunker, Boiler &amp; FGT Installation: Level 3 schedule update remains outstanding
+HDPE fire fighting pipe: ASTM-compliant pipe is not available from local suppliers in Thailand
+and may need to be imported, which could extend procurement lead time and impact
+construction schedule
+Limited site access roads may impact construction productivity and material logistics.
+Issue to request HO support:
+Drawing of Transformer Foundation Plan and Detail
+Safety &amp; Health
+Management Weekly Route Walk - Every Tuesday
+Weekly ESH Meeting - Every Tuesday
+Weekly Project Meeting with - Every Tuesday
+Toolbox Talk - Everyday before working
+Safety training (if any)
+Inspect equipment before working (Daily)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t>PRJ-020</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>PSD</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Completion of Bunker Building Concrete pouring Lift 1 Wall -5.7 to +1.0 EL ; (First step is to pour concrete up to kicker level on 26-27 Jun ; the
+second step is to pour the concrete up to +1.00 EL on 7-8 Jul
+CEEC/STECON will hand over the main 8 column pedestals (excluding the ground base slab) of the Boiler on 6th of July 2026 for HUASHI to perform
+the first lift of the steel structure on 7-JUL-2026. The remaining 4 column pedestals in the boiler area must be handed over to Huashi within 7 days
+on 14-JUL-2026 of the handover of the above columns.
+Partial handover (civil works) of Switchgear room in the STG &amp; EC Building, including all related areas required for the installation of 22 kV and 11 kV
+switchgear and power cables.
+Note : The scheduled date for the partial handover of the Switchgear Room and related areas is currently under review by CEEC. Handover schedule will be
+Increase Manpower up to 200 within June 2026
+66 Safety Weekly Audit issue status by weekly
+Total Issues
+Since 2 Jan 2026 5
+11 - 17 June
+Safety Weekly Audit issue Status Chart
+Open Closed
+Before After
+Concrete poor waste Already improved
+Government Agencies
+Problem : Electric Pole obstruct Entrance
+ต ำแหน่งเสำไฟฟ้ำเดมิ</t>
+        </is>
+      </c>
+      <c r="E19" s="16" t="inlineStr">
+        <is>
+          <t>Key Lookahead milestone:
+Bunker building : Lift 1 (-5.7 to +1 EL) First step is to pour concrete up to kicker level on 26-
+27 Jun ; the second step is to pour the concrete up to +1.00 meters on (7-8 July)
+Boiler island area : Pouring Concrete
+STG&amp;ECB : Foundation Up to ground.
+Area of Concern:
+Increase Manpower up to 200 within June 2026
+Bunker, Boiler &amp; FGT,STG Installation: Level 3 schedule update remains outstanding
+HDPE fire fighting pipe: ASTM-compliant pipe is not available from local suppliers in Thailand
+and may need to be imported, which could extend procurement lead time and impact
+construction schedule
+Issue to request HO support:
+Transformer Foundation Plan and Detail Drawings
+Concern(delay)
+Site to Monitor Increasing of Manpower
+Safety &amp; Health
+Management Weekly Route Walk - Every Tuesday
+Weekly ESH Meeting - Every Tuesday
+Weekly Project Meeting with - Every Tuesday
+Toolbox Talk - Everyday before working</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="16" t="inlineStr">
+        <is>
+          <t>PRJ-021</t>
+        </is>
+      </c>
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>PWW1</t>
+        </is>
+      </c>
+      <c r="C20" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D20" s="16" t="inlineStr">
+        <is>
+          <t>Refuse Bunker foundation construction work
+Boiler Island foundation construction
+STG Building construction
+Follow up EPC to revise the catch-up plan and monitor work progress.
+Increase overtime activities and inform neighbors about the plan.
+Expedite for Method Statement/ Engineering drawing
+Revise the catch-up plan and monitor work progress.
+Safety Weekly Audit issue status by weekly
+Total Issues 40
+Since 2 Apr 2026
+Safety Weekly Audit issue Status Chart
+April'26 May'26 4-10 Jun'26 11-17 Jun'26
+0 Open Closed
+Housekeeping
+Open Closed
+BEFORE AFTER 29
+• BOP DWG&amp;Cal. No calculation for OE to verify
+• Follow up the foundation calculation of BOP building to confirm the type of foundation. (Within 19 June 26)
+PWW Access road
+Follow up Access Road Drawing and comment Drawing.</t>
+        </is>
+      </c>
+      <c r="E20" s="16" t="inlineStr">
+        <is>
+          <t>Safety &amp; Health:
+• Safety Toolbox Talk before starting work and Mass Safety Talk.
+• Safety induction training.
+• Tools and equipment’s inspection.
+• Management walkdown.
+• Random alcohol test.
+• Random drug test.
+Environment &amp; CoP:
+• Water spray to reduce dust.
+• Wheel washing before entering public road.
+• Road cleaning.
+• Prepare for LTA&amp;ADB audit.
+Start July to end of Aug 26 • Bunker wall
+• Continuous install platform for wall 2nd step
+• Continuous backfill work
+• Start install rebar work
+• Rebar work – Lack of manpower
+Wall 2nd step to +5.45 m. (Use jump form) • Stecon allocate worker to boiler and STG building area so no manpower
+Plan 26 June 26
+for start rebar work. (Resume rebar work on 22 June 26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="16" t="inlineStr">
+        <is>
+          <t>PRJ-022</t>
+        </is>
+      </c>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>PWW2</t>
+        </is>
+      </c>
+      <c r="C21" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>Refuse Bunker foundation construction work
+Boiler Island foundation construction
+STG foundation construction
+Follow up catch up plan
+Expedite for Method Statement/ Engineering drawing
+46 Safety Weekly Audit issue status by weekly
+Total Issues
+Since 2 Apr 2026
+April'26 May'26 4-10 Jun '26 11-17 Jun'26
+Safety Weekly Audit issue Status Chart
+Open Closed
+Material storage and housekeeping.
+BEFORE AFTER
+• BOP DWG&amp;Cal. No calculation for OE to verify
+• Follow up the foundation calculation of BOP building to confirm the type of foundation. (Within 19 June 26)
+• 19 June 26: CEEC still not receive from infra.
+• Diesel oil tank need to relocation according to the permit (Setback 3.00 m.) around bun wall.
+Fire water system
+Follow up equipment(Jockey water pump and Diesel water pump). [Now status CEEC Bidding Process]
+- Follow up CEEC Order Jockey water pump and Diesel water pump.&gt;&gt;Still CEEC Biding process.</t>
+        </is>
+      </c>
+      <c r="E21" s="16" t="inlineStr">
+        <is>
+          <t>Safety &amp; Health:
+• Safety Toolbox Talk before starting work and Mass Safety Talk.
+• Safety induction training.
+• Tools and equipment’s inspection.
+• Management walkdown.
+• Random alcohol test.
+• Random drug test.
+Environment &amp; CoP:
+• Water spray to reduce dust.
+• Wheel washing before entering public road.
+• Road cleaning.
+• Prepare for LTA&amp;ADB audit.
+• Refuse bunker wall
+• Continuous rebar and formwork to 1.0 m
+Wall rebar work – 100% • Concrete pouring to 1.0 m on 23-Jun-26
+Wall formwork – 90% • Bunker building
+• Continuous Install rebar, formwork and pouring concrete surrounding column
+• The rebar detail tipping hall side not correct, must reinstall before pouring concrete.
+• The position of the columnhas been changed from the previous design. (Pending)
+Activity Qty total Qty complete %Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="16" t="inlineStr">
+        <is>
+          <t>PRJ-023</t>
+        </is>
+      </c>
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>TPP</t>
+        </is>
+      </c>
+      <c r="C22" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D22" s="16" t="inlineStr">
+        <is>
+          <t>Bunker Pit Wall to +5.45 EL
+Bunker Building ground level construction
+Boiler structure construction
+STG&amp;EC Building construction
+Underground Piping work
+Grate steel structure installation
+Ground floor level construction for Tipping Area
+Duct bank and Cathodic protection installation
+Concern (delay)
+Concrete pouring delay from additional embedded plate
+Late manufacturing for steel roof structure and cladding structure
+Construction progress delayed
+Underground pipes are required long lead for fabrication and delivery from oversea manufacturer. (Steel pipe 24”&amp;28”)
+1 Duct bank and Cathodic protection drawing were not finalized
+2 Delay of Material purchasing.
+STECON is accelerating embedded plate preparation and installation.
+Follow-up CEEC/SEPEC to urgently conclude the detail of steel roof structure and cladding structure
+SEPEC/STECON are required to expedite works
+STECON proceed to purchasing and prepare catch-up plan
+1 Follow-up the detail drawing of Duct bank and Cathodic protection in Weekly meeting.</t>
+        </is>
+      </c>
+      <c r="E22" s="16" t="inlineStr">
+        <is>
+          <t>(12 Iun 26) (19 Iun 26)
+Activities CC/SC (*)
+Plan Actual Diff. Plan Actual Diff. Acc.Plan
+% % % % % % %
+Engineering 10% 59.50 39.80 -19.70 67.58 42.52 -25.06 74.32
+Procurement 40% 68.99 65.43 -3.56 71.12 69.35 -1.77 72.89
+Construction 40% 11.51 11.39 -0.12 13.16 11.76 -1.40 14.29
+Commissioning 10% 0 0 0 0 0 0 0
+Overall 100% 38.15 34.71 -3.44 40.47 36.70 -3.77 42.30
+Safety &amp; Health :
+• Conduct SafetyToolbox Talk before starting work.
+• Mass Safety Talk at Site Area
+• Management Walk Down every Friday (10.00 – 11.00)
+• HSE Weekly Audit every Wednesday (10.00-11.00)
+• HSE Weekly Meeting with Subcontractor every Wednesday (10.00-11.00)
+• Safety Induction Training for new comers
+• Working at height Training
+Environment &amp; CoP :
+• Water spray at construction site
+• Temporary Wheel wash station</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="16" t="inlineStr">
+        <is>
+          <t>PRJ-024</t>
+        </is>
+      </c>
+      <c r="B23" s="16" t="inlineStr">
+        <is>
+          <t>TSE</t>
+        </is>
+      </c>
+      <c r="C23" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D23" s="16" t="inlineStr">
+        <is>
+          <t>Bunker and surrounding: Foundation up to ground (including the surrounding room, underground grounding system).
+Boiler : Boiler steel structure.
+Flue gas treatment : Foundation work.
+STG &amp; ECB : Foundation up to ground (including the surrounding room, underground grounding system).
+Tipping hall: Pilling work and foundation.
+Concern (delay)
+Delay finish of bunker foundations up to ground level. Target on PMS 08 May 2026.
+Delay finish of STG foundations up to ground level. Target on PMS 08 Jun 2026.
+CEEC/STECON prepared catch-up plan for bunker and follow up
+CEEC/STECON will increase man power more than plan
+- This week (Finished : 1 , Remaining : 2)
+- Total (Finished : 40 , Remaining : 2)
+1 RFC , NO NCR
+7 Stakeholder Engagement Plan Continue as plan
+8 SHE Plan for counting manpower working at site There will be generated counting manpower data report the first time on
+&lt;22 Jun 2026&gt;
+9 Status of EPC Foreigner staff and worker personal mandatory document Pending 27 prs. &lt;Plan to finish Jun 2026&gt;
+42 Safety Weekly Audit issue
+Total Issues
+(Since 2 Apr 2026 onwards) 8</t>
+        </is>
+      </c>
+      <c r="E23" s="16" t="inlineStr">
+        <is>
+          <t>Activities CC/SC (*)
+Actual Diff. Actual Diff. Acc.Plan
+Engineering 10% 75.14% 46.47% -28.47% 81.62% 48.01% -33.61% 86.57%
+Procurement 40% 75.73% 69.68% -6.05% 77.41% 74.49% -2.92% 79.32%
+Construction 40% 13.49% 12.17% -1.32% 14.79% 14.66% -0.13% 16.34%
+Commissioning 10% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00%
+Overall 100% 43.20% 37.39% -5.81% 45.04% 40.46% -4.58% 46.92%
+5 Maximum Quantity of Heavy Machinery at Site Inspection as period
+and keep related document
+6 Summary of SHE Weekly Audit issues Walk down
+- This week (Finished : 1 , Remaining : 2)
+- Total (Finished : 40 , Remaining : 2)
+1 RFC , NO NCR
+7 Stakeholder Engagement Plan Continue as plan
+8 SHE Plan for counting manpower working at site There will be generated counting manpower data report the first time on
+&lt;22 Jun 2026&gt;
+9 Status of EPC Foreigner staff and worker personal mandatory document Pending 27 prs. &lt;Plan to finish Jun 2026&gt;
+Safety &amp; Health:
+• Safety Toolbox Talk before starting work and Mass Toolbox Talk and counting manpower
+• Safety training for newcomer</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="16" t="inlineStr">
+        <is>
+          <t>PRJ-025</t>
+        </is>
+      </c>
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>Pak Lay</t>
+        </is>
+      </c>
+      <c r="C24" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D24" s="16" t="inlineStr">
+        <is>
+          <t>No. Description Progress Remark
+Contractor submitted the Contracor’s
+The contractor has appointed persons to all positions of key personnel and provided a
+representative proposal for the
+detailed organization chart to the employer before the commencement of LNTP works,
+1 Employer’s review. And key
+and for this purpose sub-clause 6.12 of the general conditions shall apply mutatis
+personnel and organization are also
+submitted for review.
+The EPC contractor has sorted out a total of 38 types of permits required for the
+contract to take effect and 33 have been completed.
+No Issue Detail Action by Target ate Progress Remark
+Harmonized Master Submit harmonized project master schedule
+1 EPC \ already done
+Schedule (P6 L4) (Primavera P6 Level 4).
+Technical Specs &amp;
+Finalize technical specs &amp; performance
+2 Performance EPC \ In progress
+guarantees for turbine &amp; generator package.
+Accelerate Design</t>
+        </is>
+      </c>
+      <c r="E24" s="16" t="inlineStr">
+        <is>
+          <t>List of Issues to be Coordinated
+Planned (%) (%) (%)
+Design Works 0.404% 14.37% 0.404% 14.772% 0.404% 15.176% 0.404% 15.580%
+Procurement,
+Production &amp; 0.386% 4.08% 0.386% 4.468% 0.386% 4.854% 0.386% 5.240%
+Preparatory
+605% 22.30% 0.605% 22.904% 0.705% 23.609% 0.705% 24.314%
+614% 17.88% 0.614% 18.493% 0.614% 19.106% 0.614% 19.720%
+Construction
+00% 0.000% 0.000% 0.000% 0.000% 0.000% 0.000%
+430% 10.68% 0.430% 11.111% 0.430% 11.541% 0.430% 11.970%
+Phase 1 &amp; 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="16" t="inlineStr">
+        <is>
+          <t>PRJ-026</t>
+        </is>
+      </c>
+      <c r="B25" s="16" t="inlineStr">
+        <is>
+          <t>Pak Beng</t>
+        </is>
+      </c>
+      <c r="C25" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D25" s="16" t="inlineStr">
+        <is>
+          <t>Discipline Qty NO.of PKG
+This Accum This Accum This Accum This Accum
+HL240 Main Batching Plant 2 44 0 44 0 44 0 44 0 44
+Chiller 3 5 0 5 0 0 0 0 0 0
+Ice Plant 3 16 0 16 16 16 16 16 0 0
+Air-cooled Main Unit 3 3 0 3 0 0 0 0 0 0
+Single-Stage Hammer Crusher 2 6 0 6 6 6 6 6 0 0
+Grizzly Feeder 2 2 0 2 0 2 0 2 0 2
+Impact Crusher 2 2 0 2 0 2 0 2 0 2
+Impact Sand Maker; High-
+1 3 0 3 0 3 0 3 0 3
+Pressure Grinding Rolls (HPGR)
+115kv Main Transformer 1 1 0 1 1 1 1 1 1 1
+115kv Tower Material 33 5 0 5 0 5 0 5 0 5
+Total 52 87 0 87 23 79 23 79 1 57
+Right bank abutment、
+Downstream Approach
+Civil 513 460 45 8 44 40 2 2 557 500 47 10
+Channel、R2 Road 、
+Spoil Disposal</t>
+        </is>
+      </c>
+      <c r="E25" s="16" t="inlineStr">
+        <is>
+          <t>Health and Safety Health and Safety
+- Ongoing conduct HSE general induction and training for
+- Ongoing conduct daily HSE toolbox meeting before
+working everyday.
+- Enforce on using basic of PPEs (safety vest, safety helmet
+and safety shoes) at working site.
+Arranged and conducted safety month promotion activities - Closely check for the project’s safety production month
+Conducted HSE toolbox meeting Installed relevant safety signages in
+before working everyday the box culvert access road
+Environment (EIA/EMMP-CP) Environment (EIA/EMMP-CP)
+- Ongoing conduct routine environmental observation/
+inspection at construction site.
+- Ongoing manage housekeeping in the construction sites.
+- Conduct blast vibration monitoring in the two nearest
+Villages of Ban HuayNgeuy and Ban PakNgeuy.
+Good-housekeeping in abutment area (right bank)
+Air (Dust &amp; Noise) Monitoring in the Batching Plant 120 area.
+S/N Construction Area Construction content Unit Design Qty. Remaining Qty. Next wk plan Qty Next wk plan % Remarks
+1 Main work
+Earthwork excavation m³ 369000 127101.00 12000 3.25%</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="17" t="inlineStr">
+        <is>
+          <t>PRJ-027</t>
+        </is>
+      </c>
+      <c r="B26" s="17" t="inlineStr">
+        <is>
+          <t>TTT</t>
+        </is>
+      </c>
+      <c r="C26" s="17" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D26" s="17" t="inlineStr"/>
+      <c r="E26" s="17" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>